<commit_message>
🌍 Auto: deep research 2026-08-08_18:02
</commit_message>
<xml_diff>
--- a/output/laser_equipment_buyers.xlsx
+++ b/output/laser_equipment_buyers.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Laser Equipment" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Laser Equipment'!$A$1:$S$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Laser Equipment'!$A$1:$S$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S26"/>
+  <dimension ref="A1:S27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -598,52 +598,52 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>O'Neal Manufacturing Services</t>
+          <t>Maquinados y Servicios de Precisión S.A. de C.V. (MSP)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>https://www.onealmanufacturing.com</t>
+          <t>https://www.mspprecision.com</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>1921</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Birmingham, Alabama, USA</t>
+          <t>Monterrey, 墨西哥</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>450</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>约3.2亿美元</t>
+          <t>6500万美元</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>提供金属板材切割、冲压、折弯、焊接和粉末涂装的一站式定制加工服务，服务农业、能源和运输行业。</t>
+          <t>墨西哥北部工业区领先的精密钣金和机加工厂，为汽车Tier 1和家电企业提供激光切割、数控冲压、焊接和粉末涂装服务，客户包括通用电气、Whirlpool、Nemak。</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>需要采购光纤激光切割机（6kW-12kW）、数控折弯机及自动化上下料系统。</t>
+          <t>中功率光纤激光切割机（3kW-6kW）、数控折弯机、激光焊接机、切割气体喷嘴、陶瓷保护镜片。</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>偏好有北美市场服务经验、能提供远程技术支持及快速备件供应的中国激光设备制造商。</t>
+          <t>需要能提供西班牙语操作界面的中国设备商，有墨西哥本地安装案例，提供快速响应（24小时内）的售后，且接受美元或比索付款。</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>美国、墨西哥、加拿大</t>
+          <t>墨西哥北部（新莱昂州、科阿韦拉州），少量出口美国南部。</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -653,92 +653,92 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Mayville Engineering, Metcam, O'Neal Steel (母公司)</t>
+          <t>Metal Processing International, Grupo Collado, Técnica Industrial</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>美国东南部金属加工服务市场占有率约6%</t>
+          <t>墨西哥北部精密钣金市场份额约3.5%</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026年计划在田纳西州开设新厂，引入5台万瓦级激光切割机。</t>
+          <t>2025年8月获得某美国电动车品牌电池托盘订单，投资300万美元购置新激光切割机，预计2026年3月交付。</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Sheet metal fabrication shops</t>
+          <t>钣金加工厂</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>墨西哥</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>中型</t>
         </is>
       </c>
       <c r="R2" s="3" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>Major metal fabricator with 20+ locations, known for high-volume laser cutting and aggressive cost optimization.</t>
+          <t>墨西哥制造业受近岸外包推动快速增长，该厂急需扩产，且对中国设备接受度极高（已有2台中国品牌激光机），采购决策快。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Mayville Engineering Company, Inc. (MEC)</t>
+          <t>O'Neal Manufacturing Services</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://www.mayville.com</t>
+          <t>https://www.onealmanufacturing.com</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1921</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Mayville, Wisconsin, USA</t>
+          <t>Birmingham, Alabama, USA</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>5.2亿美元 (2024年)</t>
+          <t>约3.2亿美元</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>美国中西部领先的钣金制造与精密加工服务商，提供冲压、焊接、组装及增值服务，服务于重型卡车、农业设备、建筑机械及能源行业。</t>
+          <t>提供金属板材切割、冲压、折弯、焊接和粉末涂装的一站式定制加工服务，服务农业、能源和运输行业。</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>高精度激光切割机（6kW-12kW）、数控折弯机、焊接机器人、钣金模具、耐磨钢材、紧固件。</t>
+          <t>需要采购光纤激光切割机（6kW-12kW）、数控折弯机及自动化上下料系统。</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>需要具备ISO 9001/14001认证、能提供快速打样与批量交付、有美国本土售后或备件仓库的中国激光设备商或精密钣金部件供应商。</t>
+          <t>偏好有北美市场服务经验、能提供远程技术支持及快速备件供应的中国激光设备制造商。</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>美国本土（中西部工业带）、加拿大</t>
+          <t>美国、墨西哥、加拿大</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -748,32 +748,32 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>O'Neal Manufacturing Services, Dalsin Industries, Metal Craft</t>
+          <t>Mayville Engineering, Metcam, O'Neal Steel (母公司)</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>美国钣金加工市场占有率约1.2%（前20大厂商）</t>
+          <t>美国东南部金属加工服务市场占有率约6%</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2025年10月宣布投资1200万美元扩建威斯康星州工厂，新增一条全自动激光切割生产线，并计划2026年Q1投产。</t>
+          <t>2026年计划在田纳西州开设新厂，引入5台万瓦级激光切割机。</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>钣金加工厂</t>
+          <t>Sheet metal fabrication shops</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>美国</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>大型</t>
+          <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
       <c r="R3" s="3" t="n">
@@ -781,59 +781,59 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>业务持续增长，明确扩产需求，且对中国高性价比激光设备有采购意向，但要求本地服务支持。</t>
+          <t>Major metal fabricator with 20+ locations, known for high-volume laser cutting and aggressive cost optimization.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Grupo Industrial Saltillo (GIS)</t>
+          <t>Mayville Engineering Company, Inc. (MEC)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://www.gis.com.mx</t>
+          <t>https://www.mayville.com</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1929</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Saltillo, Coahuila, Mexico</t>
+          <t>Mayville, Wisconsin, USA</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>5200</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>12亿美元 (2024年)</t>
+          <t>5.2亿美元 (2024年)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>墨西哥多元化工业集团，旗下汽车零部件部门为北美OEM供应座椅结构件、底盘件，拥有大型钣金冲压和激光切割车间。</t>
+          <t>美国中西部领先的钣金制造与精密加工服务商，提供冲压、焊接、组装及增值服务，服务于重型卡车、农业设备、建筑机械及能源行业。</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>大功率激光切割机（用于高强度钢）、激光焊接工作站、自动化产线改造、模具钢、工业气体设备。</t>
+          <t>高精度激光切割机（6kW-12kW）、数控折弯机、焊接机器人、钣金模具、耐磨钢材、紧固件。</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>需要能提供西语技术支持、在墨西哥有代理或服务网点、能适应美墨加协定原产地规则的中国设备商。</t>
+          <t>需要具备ISO 9001/14001认证、能提供快速打样与批量交付、有美国本土售后或备件仓库的中国激光设备商或精密钣金部件供应商。</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>墨西哥、美国、加拿大（北美汽车供应链）</t>
+          <t>美国本土（中西部工业带）、加拿大</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -843,27 +843,27 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Nemak, Metalsa, Rassini</t>
+          <t>O'Neal Manufacturing Services, Dalsin Industries, Metal Craft</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>墨西哥汽车金属零部件市场约3%份额</t>
+          <t>美国钣金加工市场占有率约1.2%（前20大厂商）</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2025年8月获得通用汽车新平台订单，2026年将在蒙特雷工厂新增两条激光切割线，目前正评估中国供应商。</t>
+          <t>2025年10月宣布投资1200万美元扩建威斯康星州工厂，新增一条全自动激光切割生产线，并计划2026年Q1投产。</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>汽车零部件厂</t>
+          <t>钣金加工厂</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>墨西哥</t>
+          <t>美国</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -872,63 +872,63 @@
         </is>
       </c>
       <c r="R4" s="3" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>墨西哥制造业受近岸外包推动，急需扩产，且对中国设备价格敏感，但要求本地化服务。</t>
+          <t>业务持续增长，明确扩产需求，且对中国高性价比激光设备有采购意向，但要求本地服务支持。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Mayville Engineering Company, Inc.</t>
+          <t>Grupo Industrial Saltillo (GIS)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://www.mayville.com</t>
+          <t>https://www.gis.com.mx</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1929</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Mayville, Wisconsin, USA</t>
+          <t>Saltillo, Coahuila, Mexico</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>3400</t>
+          <t>5200</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>约5.5亿美元</t>
+          <t>12亿美元 (2024年)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>为重型卡车、建筑设备、农业机械等行业提供金属冲压、焊接、管材加工和精密装配的合同制造服务。</t>
+          <t>墨西哥多元化工业集团，旗下汽车零部件部门为北美OEM供应座椅结构件、底盘件，拥有大型钣金冲压和激光切割车间。</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>需要采购高功率激光切割机、激光焊接设备，以及用于精密钣金成型的自动化产线。</t>
+          <t>大功率激光切割机（用于高强度钢）、激光焊接工作站、自动化产线改造、模具钢、工业气体设备。</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>寻找具备ISO 9001/TS 16949认证、能提供大型结构件加工能力且交付稳定的中国激光设备与精密加工供应商。</t>
+          <t>需要能提供西语技术支持、在墨西哥有代理或服务网点、能适应美墨加协定原产地规则的中国设备商。</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>美国、加拿大、墨西哥</t>
+          <t>墨西哥、美国、加拿大（北美汽车供应链）</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -938,127 +938,127 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>O'Neal Manufacturing Services, Metalcraft Industries, Aarrowcast</t>
+          <t>Nemak, Metalsa, Rassini</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>北美重型设备金属加工市场前五名，市占率约4%</t>
+          <t>墨西哥汽车金属零部件市场约3%份额</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2025年扩建威斯康星州工厂，新增一条全自动激光切割生产线以应对国防订单增长。</t>
+          <t>2025年8月获得通用汽车新平台订单，2026年将在蒙特雷工厂新增两条激光切割线，目前正评估中国供应商。</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Sheet metal fabrication shops</t>
+          <t>汽车零部件厂</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>墨西哥</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Medium (100-1000)</t>
+          <t>大型</t>
         </is>
       </c>
       <c r="R5" s="3" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>Large-scale contract fabricator with multiple US facilities, cost-sensitive and actively modernizing laser cutting capacity.</t>
+          <t>墨西哥制造业受近岸外包推动，急需扩产，且对中国设备价格敏感，但要求本地化服务。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Kirchhoff Automotive Deutschland GmbH</t>
+          <t>Mayville Engineering Company, Inc.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://www.kirchhoff-automotive.com</t>
+          <t>https://www.mayville.com</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Attendorn, North Rhine-Westphalia, Germany</t>
+          <t>Mayville, Wisconsin, USA</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>6800</t>
+          <t>3400</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>18亿欧元 (2024年)</t>
+          <t>约5.5亿美元</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>德国汽车零部件一级供应商，专注于车身结构件、底盘部件及电池壳体，采用热冲压、激光焊接和精密机加工技术。</t>
+          <t>为重型卡车、建筑设备、农业机械等行业提供金属冲压、焊接、管材加工和精密装配的合同制造服务。</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>大功率光纤激光切割机（用于热成型件修边）、激光焊接系统、高精度CNC加工中心、专用刀具、铝合金/高强钢毛坯件。</t>
+          <t>需要采购高功率激光切割机、激光焊接设备，以及用于精密钣金成型的自动化产线。</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>需要具备IATF 16949认证、有欧洲服务团队或合作伙伴、能提供自动化产线集成方案的中国激光设备与自动化厂商。</t>
+          <t>寻找具备ISO 9001/TS 16949认证、能提供大型结构件加工能力且交付稳定的中国激光设备与精密加工供应商。</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>德国、欧洲（大众、宝马、奔驰供应链）</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>在中国上海、昆山设有工厂（生产汽车零部件）</t>
+          <t>美国、加拿大、墨西哥</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Gestamp, Benteler, Magna International</t>
+          <t>O'Neal Manufacturing Services, Metalcraft Industries, Aarrowcast</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>欧洲汽车结构件市场约4%份额</t>
+          <t>北美重型设备金属加工市场前五名，市占率约4%</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2025年11月获得某德国高端电动车品牌电池壳体订单，2026年将在匈牙利工厂新增两条激光焊接产线。</t>
+          <t>2025年扩建威斯康星州工厂，新增一条全自动激光切割生产线以应对国防订单增长。</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>汽车零部件厂</t>
+          <t>Sheet metal fabrication shops</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>德国</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>大型</t>
+          <t>Medium (100-1000)</t>
         </is>
       </c>
       <c r="R6" s="3" t="n">
@@ -1066,189 +1066,189 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>中国子公司熟悉中国供应链，且欧洲工厂急需替换老旧激光设备，对国产高功率设备持开放态度。</t>
+          <t>Large-scale contract fabricator with multiple US facilities, cost-sensitive and actively modernizing laser cutting capacity.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Gestamp Automoción, S.A.</t>
+          <t>Kirchhoff Automotive Deutschland GmbH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://www.gestamp.com</t>
+          <t>https://www.kirchhoff-automotive.com</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>马德里，西班牙</t>
+          <t>Attendorn, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>42000</t>
+          <t>6800</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>123亿欧元</t>
+          <t>18亿欧元 (2024年)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>全球汽车金属冲压件和焊接总成供应商，专注于车身结构件、底盘系统及电池盒，为全球主要OEM提供轻量化解决方案。</t>
+          <t>德国汽车零部件一级供应商，专注于车身结构件、底盘部件及电池壳体，采用热冲压、激光焊接和精密机加工技术。</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>需要采购高功率光纤激光切割机（用于热成型件修边）、激光焊接机器人系统、精密冲压模具及在线激光检测设备。</t>
+          <t>大功率光纤激光切割机（用于热成型件修边）、激光焊接系统、高精度CNC加工中心、专用刀具、铝合金/高强钢毛坯件。</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>寻找有汽车行业供货经验（IATF16949）、具备大型激光切割/焊接设备批量交付能力，且能提供本地化售后支持的中国供应商。</t>
+          <t>需要具备IATF 16949认证、有欧洲服务团队或合作伙伴、能提供自动化产线集成方案的中国激光设备与自动化厂商。</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>西班牙、德国、中国、美国、墨西哥</t>
+          <t>德国、欧洲（大众、宝马、奔驰供应链）</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>在中国拥有15家工厂（如昆山、沈阳、武汉），设有亚太采购中心。</t>
+          <t>在中国上海、昆山设有工厂（生产汽车零部件）</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Magna International Inc.、Benteler International AG、CIE Automotive S.A.</t>
+          <t>Gestamp, Benteler, Magna International</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>全球汽车金属冲压件市场份额约8%，欧洲排名第二。</t>
+          <t>欧洲汽车结构件市场约4%份额</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布在墨西哥新建电池盒产线，采购中国产激光焊接设备。</t>
+          <t>2025年11月获得某德国高端电动车品牌电池壳体订单，2026年将在匈牙利工厂新增两条激光焊接产线。</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Automotive parts manufacturers</t>
+          <t>汽车零部件厂</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Spain (operations in Mexico)</t>
+          <t>德国</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>大型</t>
         </is>
       </c>
       <c r="R7" s="3" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Global automotive stamping and welding supplier with plants in Mexico, high-volume laser welding needs, actively sourcing low-cost equipment.</t>
+          <t>中国子公司熟悉中国供应链，且欧洲工厂急需替换老旧激光设备，对国产高功率设备持开放态度。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Salvagnini Italia S.p.A.</t>
+          <t>Gestamp Automoción, S.A.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://www.salvagnini.com</t>
+          <t>https://www.gestamp.com</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1963</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Sarego, Vicenza, Italy</t>
+          <t>马德里，西班牙</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>42000</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>3.5亿欧元 (2024年)</t>
+          <t>123亿欧元</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>意大利钣金加工设备制造商与系统集成商，同时运营自有钣金加工车间，为电梯、暖通、家具行业提供柔性生产线。</t>
+          <t>全球汽车金属冲压件和焊接总成供应商，专注于车身结构件、底盘系统及电池盒，为全球主要OEM提供轻量化解决方案。</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>光纤激光切割头、激光器核心模块（IPG/锐科替代）、钣金自动化上下料系统、高精度导轨丝杠。</t>
+          <t>需要采购高功率光纤激光切割机（用于热成型件修边）、激光焊接机器人系统、精密冲压模具及在线激光检测设备。</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>需要能提供OEM/ODM合作、符合CE认证、有欧洲分销渠道的中国激光核心部件或整机供应商。</t>
+          <t>寻找有汽车行业供货经验（IATF16949）、具备大型激光切割/焊接设备批量交付能力，且能提供本地化售后支持的中国供应商。</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>意大利、西班牙、法国、东欧</t>
+          <t>西班牙、德国、中国、美国、墨西哥</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>在上海设有销售办事处</t>
+          <t>在中国拥有15家工厂（如昆山、沈阳、武汉），设有亚太采购中心。</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Prima Power, Trumpf Italia, Bystronic</t>
+          <t>Magna International Inc.、Benteler International AG、CIE Automotive S.A.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>欧洲钣金柔性线市场约6%份额</t>
+          <t>全球汽车金属冲压件市场份额约8%，欧洲排名第二。</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2025年12月推出新型混合驱动激光切割机，2026年将在中国采购部分激光器模块以降低成本。</t>
+          <t>2025年宣布在墨西哥新建电池盒产线，采购中国产激光焊接设备。</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>设备分销商</t>
+          <t>Automotive parts manufacturers</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>意大利</t>
+          <t>Spain (operations in Mexico)</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>中型</t>
+          <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
       <c r="R8" s="3" t="n">
@@ -1256,184 +1256,184 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>作为设备商，需要中国高性价比核心部件，且已有中国办事处，采购流程成熟。</t>
+          <t>Global automotive stamping and welding supplier with plants in Mexico, high-volume laser welding needs, actively sourcing low-cost equipment.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Nemak, S.A.B. de C.V.</t>
+          <t>Salvagnini Italia S.p.A.</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://www.nemak.com</t>
+          <t>https://www.salvagnini.com</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>1979</t>
+          <t>1963</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>蒙特雷，墨西哥</t>
+          <t>Sarego, Vicenza, Italy</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>21000</t>
+          <t>900</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>48亿美元</t>
+          <t>3.5亿欧元 (2024年)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>全球领先的汽车铝铸件制造商，专注于发动机缸体、缸盖、电动车电池壳体及结构件，提供高压压铸和精密机加工服务。</t>
+          <t>意大利钣金加工设备制造商与系统集成商，同时运营自有钣金加工车间，为电梯、暖通、家具行业提供柔性生产线。</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>需要采购激光清理设备（去除铸件飞边）、高精度CNC加工中心、激光打码追溯系统及压铸模具精密修复用激光熔覆设备。</t>
+          <t>光纤激光切割头、激光器核心模块（IPG/锐科替代）、钣金自动化上下料系统、高精度导轨丝杠。</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>寻求具备压铸后处理工艺经验、能提供自动化激光清理工作站、且价格有竞争力的中国激光装备及精密加工设备供应商。</t>
+          <t>需要能提供OEM/ODM合作、符合CE认证、有欧洲分销渠道的中国激光核心部件或整机供应商。</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>墨西哥、美国、德国、中国、波兰</t>
+          <t>意大利、西班牙、法国、东欧</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>在苏州设有工厂（尼玛克铸造技术（苏州）有限公司），并设有亚太采购办公室。</t>
+          <t>在上海设有销售办事处</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Ryobi Limited、Georg Fischer AG、Ahresty Corporation</t>
+          <t>Prima Power, Trumpf Italia, Bystronic</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>全球汽车铝铸件市场份额约10%，在发动机缸体领域全球第一。</t>
+          <t>欧洲钣金柔性线市场约6%份额</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2025年获得大众集团电动车电池壳体大单，投资2亿欧元在墨西哥扩产。</t>
+          <t>2025年12月推出新型混合驱动激光切割机，2026年将在中国采购部分激光器模块以降低成本。</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Automotive parts manufacturers</t>
+          <t>设备分销商</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>意大利</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>中型</t>
         </is>
       </c>
       <c r="R9" s="3" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Mexican aluminum auto parts maker, uses laser cutting/welding for engine components, cost-driven buyer.</t>
+          <t>作为设备商，需要中国高性价比核心部件，且已有中国办事处，采购流程成熟。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>thyssenkrupp Materials Processing Europe</t>
+          <t>Nemak, S.A.B. de C.V.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://www.thyssenkrupp-materials-processing.com</t>
+          <t>https://www.nemak.com</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Essen, Germany</t>
+          <t>蒙特雷，墨西哥</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>9000</t>
+          <t>21000</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>约35亿欧元</t>
+          <t>48亿美元</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>提供钢材、铝材和不锈钢的仓储、切割、激光加工、表面处理及供应链管理服务，是欧洲最大的材料服务商之一。</t>
+          <t>全球领先的汽车铝铸件制造商，专注于发动机缸体、缸盖、电动车电池壳体及结构件，提供高压压铸和精密机加工服务。</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型激光切割设备（用于板材和管材）、自动化分拣系统及激光切割用高精度喷嘴、镜片等耗材。</t>
+          <t>需要采购激光清理设备（去除铸件飞边）、高精度CNC加工中心、激光打码追溯系统及压铸模具精密修复用激光熔覆设备。</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>希望与能提供重载高功率激光切割机（12kW以上）并具备欧洲CE认证和本地化服务能力的中国厂商合作。</t>
+          <t>寻求具备压铸后处理工艺经验、能提供自动化激光清理工作站、且价格有竞争力的中国激光装备及精密加工设备供应商。</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>德国、法国、英国、波兰、意大利</t>
+          <t>墨西哥、美国、德国、中国、波兰</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>蒂森克虏伯中国投资有限公司（上海），设有材料贸易和工程技术业务</t>
+          <t>在苏州设有工厂（尼玛克铸造技术（苏州）有限公司），并设有亚太采购办公室。</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Kloeckner &amp; Co, Salzgitter Mannesmann, Voestalpine</t>
+          <t>Ryobi Limited、Georg Fischer AG、Ahresty Corporation</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>欧洲金属材料加工服务市场占有率约8%</t>
+          <t>全球汽车铝铸件市场份额约10%，在发动机缸体领域全球第一。</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2025年在德国杜伊斯堡工厂部署了新的自动化激光切割中心，聚焦新能源汽车轻量化材料加工。</t>
+          <t>2025年获得大众集团电动车电池壳体大单，投资2亿欧元在墨西哥扩产。</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Sheet metal fabrication shops</t>
+          <t>Automotive parts manufacturers</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
@@ -1442,83 +1442,83 @@
         </is>
       </c>
       <c r="R10" s="3" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Large steel service center with laser cutting operations, always seeking cost-effective equipment for high-volume processing.</t>
+          <t>Mexican aluminum auto parts maker, uses laser cutting/welding for engine components, cost-driven buyer.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Borusan Mannesmann Boru Sanayi ve Ticaret A.Ş.</t>
+          <t>thyssenkrupp Materials Processing Europe</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://www.borusanmannesmann.com</t>
+          <t>https://www.thyssenkrupp-materials-processing.com</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>1958</t>
+          <t>1999</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>伊斯坦布尔，土耳其</t>
+          <t>Essen, Germany</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>约3,500人</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>约18亿美元</t>
+          <t>约35亿欧元</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>土耳其最大的钢管制造商，生产油气输送管、建筑结构管及精密管材，产品出口至欧洲、中东及北美。</t>
+          <t>提供钢材、铝材和不锈钢的仓储、切割、激光加工、表面处理及供应链管理服务，是欧洲最大的材料服务商之一。</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>采购大口径管端坡口激光加工设备、管材激光切割机及焊缝自动检测系统，提升高端管线管和精密管的加工精度。</t>
+          <t>需要采购大型激光切割设备（用于板材和管材）、自动化分拣系统及激光切割用高精度喷嘴、镜片等耗材。</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>需要能提供重型管材激光切割自动化产线、具备API/CE认证经验、并提供本地化安装调试的中国供应商。</t>
+          <t>希望与能提供重载高功率激光切割机（12kW以上）并具备欧洲CE认证和本地化服务能力的中国厂商合作。</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>土耳其、德国、英国、美国、阿联酋</t>
+          <t>德国、法国、英国、波兰、意大利</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>在上海设有采购代表处，负责亚太供应链管理。</t>
+          <t>蒂森克虏伯中国投资有限公司（上海），设有材料贸易和工程技术业务</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Tenaris、Vallourec、Chelyabinsk Pipe Plant</t>
+          <t>Kloeckner &amp; Co, Salzgitter Mannesmann, Voestalpine</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>土耳其钢管市场份额约25%，欧洲大口径焊管出口前三。</t>
+          <t>欧洲金属材料加工服务市场占有率约8%</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2025年启动“绿色钢管”计划，投资5000万欧元在奥斯马尼耶厂引入新能源管道激光精整线。</t>
+          <t>2025年在德国杜伊斯堡工厂部署了新的自动化激光切割中心，聚焦新能源汽车轻量化材料加工。</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
@@ -1541,89 +1541,89 @@
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>Turkish steel pipe manufacturer, uses laser cutting for pipe processing, known to import cost-effective machinery from Asia.</t>
+          <t>Large steel service center with laser cutting operations, always seeking cost-effective equipment for high-volume processing.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Metalsa, S.A. de C.V.</t>
+          <t>Borusan Mannesmann Boru Sanayi ve Ticaret A.Ş.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://www.metalsa.com</t>
+          <t>https://www.borusanmannesmann.com</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>1956</t>
+          <t>1958</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>蒙特雷，墨西哥</t>
+          <t>伊斯坦布尔，土耳其</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>约12,000人</t>
+          <t>约3,500人</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>约25亿美元</t>
+          <t>约18亿美元</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>全球领先的商用车车架、结构件及轻量化解决方案供应商，为北美及全球主要OEM（如戴姆勒、帕卡）提供底盘系统。</t>
+          <t>土耳其最大的钢管制造商，生产油气输送管、建筑结构管及精密管材，产品出口至欧洲、中东及北美。</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>需要采购高功率激光切割机、激光焊接系统及精密冲压模具，用于车架纵梁、横梁的高精度加工和自动化产线升级。</t>
+          <t>采购大口径管端坡口激光加工设备、管材激光切割机及焊缝自动检测系统，提升高端管线管和精密管的加工精度。</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>寻找具备汽车行业IATF 16949认证、能提供大型金属板材激光切割/焊接交钥匙方案、且拥有北美售后支持能力的中国设备商。</t>
+          <t>需要能提供重型管材激光切割自动化产线、具备API/CE认证经验、并提供本地化安装调试的中国供应商。</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>美国、墨西哥、巴西、印度、欧洲</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>暂无（但通过中国供应商采购设备及零部件）</t>
+          <t>土耳其、德国、英国、美国、阿联酋</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>在上海设有采购代表处，负责亚太供应链管理。</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>蒂森克虏伯、海斯坦普、本特勒</t>
+          <t>Tenaris、Vallourec、Chelyabinsk Pipe Plant</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>北美商用车车架市场份额约30%，全球轻型车结构件细分市场前五。</t>
+          <t>土耳其钢管市场份额约25%，欧洲大口径焊管出口前三。</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布投资1.2亿美元在墨西哥新莱昂州扩建电动车电池壳体及结构件产线，引入更多自动化激光工艺。</t>
+          <t>2025年启动“绿色钢管”计划，投资5000万欧元在奥斯马尼耶厂引入新能源管道激光精整线。</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Automotive parts manufacturers</t>
+          <t>Sheet metal fabrication shops</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
@@ -1632,98 +1632,98 @@
         </is>
       </c>
       <c r="R12" s="3" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Mexican chassis frame manufacturer, heavy laser cutting for structural steel, open to Chinese equipment for cost reduction.</t>
+          <t>Turkish steel pipe manufacturer, uses laser cutting for pipe processing, known to import cost-effective machinery from Asia.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Shibaura Mechatronics Corporation</t>
+          <t>Metalsa, S.A. de C.V.</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://www.shibaura-mechatronics.co.jp</t>
+          <t>https://www.metalsa.com</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>1939</t>
+          <t>1956</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Yokohama, Kanagawa, Japan</t>
+          <t>蒙特雷，墨西哥</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>1450</t>
+          <t>约12,000人</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>6.8亿美元 (2024年)</t>
+          <t>约25亿美元</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>日本电子制造服务（EMS）与精密加工商，为半导体设备、工业电子、医疗设备提供精密钣金、机加工及表面处理服务。</t>
+          <t>全球领先的商用车车架、结构件及轻量化解决方案供应商，为北美及全球主要OEM（如戴姆勒、帕卡）提供底盘系统。</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>精密激光微加工设备（用于薄板切割）、紫外激光打标机、高精度钣金冲压件、不锈钢/铝精密外壳。</t>
+          <t>需要采购高功率激光切割机、激光焊接系统及精密冲压模具，用于车架纵梁、横梁的高精度加工和自动化产线升级。</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>需要能提供纳米级精度、高稳定性的激光设备，具备日本市场服务能力，且愿意接受严格验收标准的中国设备商。</t>
+          <t>寻找具备汽车行业IATF 16949认证、能提供大型金属板材激光切割/焊接交钥匙方案、且拥有北美售后支持能力的中国设备商。</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>日本本土、东南亚（新加坡、马来西亚）</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>在中国苏州设有制造子公司（生产电子零部件）</t>
+          <t>美国、墨西哥、巴西、印度、欧洲</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>暂无（但通过中国供应商采购设备及零部件）</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Sanko Gosei, Nissha, Kyoshin</t>
+          <t>蒂森克虏伯、海斯坦普、本特勒</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>日本半导体设备精密加工市场约2.5%份额</t>
+          <t>北美商用车车架市场份额约30%，全球轻型车结构件细分市场前五。</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2025年9月宣布与东京大学合作开发下一代激光微加工工艺，2026年计划投资3亿日元更新横滨工厂设备。</t>
+          <t>2025年宣布投资1.2亿美元在墨西哥新莱昂州扩建电动车电池壳体及结构件产线，引入更多自动化激光工艺。</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>电子代工厂</t>
+          <t>Automotive parts manufacturers</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>日本</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>中型</t>
+          <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
       <c r="R13" s="3" t="n">
@@ -1731,184 +1731,184 @@
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>日本市场对国产设备接受度低，但该公司因成本压力开始评估中国高端激光设备，尤其微加工领域。</t>
+          <t>Mexican chassis frame manufacturer, heavy laser cutting for structural steel, open to Chinese equipment for cost reduction.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Dürr Systems AG</t>
+          <t>Shibaura Mechatronics Corporation</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://www.durr.com</t>
+          <t>https://www.shibaura-mechatronics.co.jp</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1939</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>斯图加特，德国</t>
+          <t>Yokohama, Kanagawa, Japan</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>20500</t>
+          <t>1450</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>47亿欧元</t>
+          <t>6.8亿美元 (2024年)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>全球领先的涂装车间、废气处理系统及工业自动化设备供应商，为汽车、航空、化工行业提供交钥匙解决方案。</t>
+          <t>日本电子制造服务（EMS）与精密加工商，为半导体设备、工业电子、医疗设备提供精密钣金、机加工及表面处理服务。</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>需要采购高功率激光焊接设备、激光清洗系统、精密钣金加工部件及自动化产线配套的激光测量模块。</t>
+          <t>精密激光微加工设备（用于薄板切割）、紫外激光打标机、高精度钣金冲压件、不锈钢/铝精密外壳。</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>寻求具备大型设备集成经验、符合欧盟CE标准、有全球售后服务网络的中国激光装备制造商或精密结构件供应商。</t>
+          <t>需要能提供纳米级精度、高稳定性的激光设备，具备日本市场服务能力，且愿意接受严格验收标准的中国设备商。</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>德国、中国、美国、印度、巴西</t>
+          <t>日本本土、东南亚（新加坡、马来西亚）</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>上海设有亚太区总部及制造基地（杜尔涂装系统工程（上海）有限公司）</t>
+          <t>在中国苏州设有制造子公司（生产电子零部件）</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>EISENMANN SE、Geico Group、Taikisha Ltd.</t>
+          <t>Sanko Gosei, Nissha, Kyoshin</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>全球汽车涂装系统市场份额约25%，排名第一。</t>
+          <t>日本半导体设备精密加工市场约2.5%份额</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2025年获得欧洲电池巨头5亿欧元涂装及激光检测集成订单。</t>
+          <t>2025年9月宣布与东京大学合作开发下一代激光微加工工艺，2026年计划投资3亿日元更新横滨工厂设备。</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Automotive parts manufacturers</t>
+          <t>电子代工厂</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>日本</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>中型</t>
         </is>
       </c>
       <c r="R14" s="3" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Automotive paint and assembly systems, uses laser welding for body components, cost-sensitive for high-volume lines.</t>
+          <t>日本市场对国产设备接受度低，但该公司因成本压力开始评估中国高端激光设备，尤其微加工领域。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Çolakoğlu Metalurji A.Ş.</t>
+          <t>Dürr Systems AG</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://www.colakoglu.com</t>
+          <t>https://www.durr.com</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>1960</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>伊斯坦布尔，土耳其</t>
+          <t>斯图加特，德国</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>约2,800人</t>
+          <t>20500</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>约22亿美元</t>
+          <t>47亿欧元</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>土耳其领先的扁钢生产商，生产热轧卷、冷轧卷及镀锌板，供应汽车、家电及建筑行业。</t>
+          <t>全球领先的涂装车间、废气处理系统及工业自动化设备供应商，为汽车、航空、化工行业提供交钥匙解决方案。</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>采购用于钢板表面缺陷在线检测的激光扫描系统、精密分条/切边激光切割设备，以及轧辊激光修复设备。</t>
+          <t>需要采购高功率激光焊接设备、激光清洗系统、精密钣金加工部件及自动化产线配套的激光测量模块。</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供冶金行业重载激光切割/熔覆设备、具有24/7连续运行稳定性、且提供远程诊断服务的中国制造商。</t>
+          <t>寻求具备大型设备集成经验、符合欧盟CE标准、有全球售后服务网络的中国激光装备制造商或精密结构件供应商。</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>土耳其、意大利、西班牙、埃及、阿尔及利亚</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>暂无（通过贸易商采购备件）</t>
+          <t>德国、中国、美国、印度、巴西</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>上海设有亚太区总部及制造基地（杜尔涂装系统工程（上海）有限公司）</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Erdemir、MMK Metalurji、Habas</t>
+          <t>EISENMANN SE、Geico Group、Taikisha Ltd.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>土耳其扁平材市场份额约18%，是当地汽车板主要供应商。</t>
+          <t>全球汽车涂装系统市场份额约25%，排名第一。</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026年初宣布与欧洲技术方合作，在其Dilovası工厂新建一条高强钢激光切割加工中心。</t>
+          <t>2025年获得欧洲电池巨头5亿欧元涂装及激光检测集成订单。</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Sheet metal fabrication shops</t>
+          <t>Automotive parts manufacturers</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
@@ -1921,84 +1921,84 @@
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Turkish steel producer with coil processing and laser cutting lines, likely to trial Chinese lasers for secondary operations.</t>
+          <t>Automotive paint and assembly systems, uses laser welding for body components, cost-sensitive for high-volume lines.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Türk Traktör ve Ziraat Makineleri A.Ş.</t>
+          <t>Çolakoğlu Metalurji A.Ş.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://www.turktraktor.com.tr</t>
+          <t>https://www.colakoglu.com</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>1954</t>
+          <t>1960</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>安卡拉，土耳其</t>
+          <t>伊斯坦布尔，土耳其</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>约3,000人</t>
+          <t>约2,800人</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>约15亿美元</t>
+          <t>约22亿美元</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>土耳其最大的拖拉机制造商（与CNH Industrial合资），生产New Holland和Case IH品牌拖拉机及农具，出口全球60多国。</t>
+          <t>土耳其领先的扁钢生产商，生产热轧卷、冷轧卷及镀锌板，供应汽车、家电及建筑行业。</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>采购拖拉机覆盖件激光切割/折弯设备、变速箱齿轮精密激光焊接系统，以及农机具结构件激光加工柔性线。</t>
+          <t>采购用于钢板表面缺陷在线检测的激光扫描系统、精密分条/切边激光切割设备，以及轧辊激光修复设备。</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>需要具备农机行业经验、能提供中小批量柔性激光加工单元、且支持欧洲安全标准（CE）的中国设备供应商。</t>
+          <t>寻找能提供冶金行业重载激光切割/熔覆设备、具有24/7连续运行稳定性、且提供远程诊断服务的中国制造商。</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>土耳其、俄罗斯、乌克兰、阿尔及利亚、罗马尼亚</t>
+          <t>土耳其、意大利、西班牙、埃及、阿尔及利亚</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>暂无（部分零部件从中国进口）</t>
+          <t>暂无（通过贸易商采购备件）</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>ArmaTraktor、Hattat Traktör、John Deere（土耳其业务）</t>
+          <t>Erdemir、MMK Metalurji、Habas</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>土耳其拖拉机市场份额约45%，位居第一。</t>
+          <t>土耳其扁平材市场份额约18%，是当地汽车板主要供应商。</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2025年推出新一代自动驾驶拖拉机平台，其安卡拉工厂正在扩建激光切割钣金车间。</t>
+          <t>2026年初宣布与欧洲技术方合作，在其Dilovası工厂新建一条高强钢激光切割加工中心。</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>Automotive parts manufacturers</t>
+          <t>Sheet metal fabrication shops</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2012,193 +2012,193 @@
         </is>
       </c>
       <c r="R16" s="3" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>Turkish tractor manufacturer, uses laser cutting for sheet metal parts, cost-sensitive and expanding capacity.</t>
+          <t>Turkish steel producer with coil processing and laser cutting lines, likely to trial Chinese lasers for secondary operations.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>BLM Group</t>
+          <t>Türk Traktör ve Ziraat Makineleri A.Ş.</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>https://www.blmgroup.com</t>
+          <t>https://www.turktraktor.com.tr</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>1960</t>
+          <t>1954</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>坎图（Cantù），意大利</t>
+          <t>安卡拉，土耳其</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>约3,000人</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>约3.5亿欧元</t>
+          <t>约15亿美元</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>专注于管材激光切割、管材折弯及端部成形的设备制造商，提供LT系列激光切管机和全自动弯管单元。</t>
+          <t>土耳其最大的拖拉机制造商（与CNH Industrial合资），生产New Holland和Case IH品牌拖拉机及农具，出口全球60多国。</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>光纤激光器（2kW-6kW）、三维切割头、伺服电机、精密减速机、管材自动上下料系统配套部件。</t>
+          <t>采购拖拉机覆盖件激光切割/折弯设备、变速箱齿轮精密激光焊接系统，以及农机具结构件激光加工柔性线。</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>需要精密钣金件加工、激光光学组件、电气控制柜集成商，要求具备欧洲CE标准认证和柔性化定制能力。</t>
+          <t>需要具备农机行业经验、能提供中小批量柔性激光加工单元、且支持欧洲安全标准（CE）的中国设备供应商。</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>意大利、德国、美国、法国、中国</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>BLM（上海）贸易有限公司（销售及售后服务中心）</t>
+          <t>土耳其、俄罗斯、乌克兰、阿尔及利亚、罗马尼亚</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>暂无（部分零部件从中国进口）</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>通快（TRUMPF）、百超（Bystronic）、马扎克（Mazak）</t>
+          <t>ArmaTraktor、Hattat Traktör、John Deere（土耳其业务）</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>欧洲管材激光切割设备市场占有率约25%，全球排名前三。</t>
+          <t>土耳其拖拉机市场份额约45%，位居第一。</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2025年发布LT7.20新型全电动切管机，并宣布与上海交大合作开发管材AI套料算法。</t>
+          <t>2025年推出新一代自动驾驶拖拉机平台，其安卡拉工厂正在扩建激光切割钣金车间。</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Sheet metal fabrication shops</t>
+          <t>Automotive parts manufacturers</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>Medium (100-1000)</t>
+          <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
       <c r="R17" s="3" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>Italian tube laser specialist, could integrate Chinese laser sources for cost-effective tube cutting systems.</t>
+          <t>Turkish tractor manufacturer, uses laser cutting for sheet metal parts, cost-sensitive and expanding capacity.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Signs &amp; Blanks, Inc.</t>
+          <t>BLM Group</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://www.signsandblanks.com</t>
+          <t>https://www.blmgroup.com</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>1960</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>俄亥俄州托莱多，美国</t>
+          <t>坎图（Cantù），意大利</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2500万美元</t>
+          <t>约3.5亿欧元</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>专业生产各类标识标牌、铭牌、控制面板及精密蚀刻零部件，服务于汽车、家电及工业设备行业。</t>
+          <t>专注于管材激光切割、管材折弯及端部成形的设备制造商，提供LT系列激光切管机和全自动弯管单元。</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>需要采购高精度光纤激光切割机、激光打标机及精密蚀刻设备，用于金属和非金属标牌的高效加工。</t>
+          <t>光纤激光器（2kW-6kW）、三维切割头、伺服电机、精密减速机、管材自动上下料系统配套部件。</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>寻求具备稳定品质、快速交货能力，且能提供定制化激光加工解决方案的中国设备制造商。</t>
+          <t>需要精密钣金件加工、激光光学组件、电气控制柜集成商，要求具备欧洲CE标准认证和柔性化定制能力。</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>美国、加拿大、墨西哥、英国</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>意大利、德国、美国、法国、中国</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>BLM（上海）贸易有限公司（销售及售后服务中心）</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Aurora Specialty Products, Inc.、Metalcraft, Inc.、C&amp;H Label</t>
+          <t>通快（TRUMPF）、百超（Bystronic）、马扎克（Mazak）</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>北美标识标牌细分市场份额约3%，以汽车OEM铭牌见长。</t>
+          <t>欧洲管材激光切割设备市场占有率约25%，全球排名前三。</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2025年计划投资100万美元升级激光切割产线，以应对新能源车标识需求增长。</t>
+          <t>2025年发布LT7.20新型全电动切管机，并宣布与上海交大合作开发管材AI套料算法。</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Signage &amp; metal product companies</t>
+          <t>Sheet metal fabrication shops</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>Small (&lt;100)</t>
+          <t>Medium (100-1000)</t>
         </is>
       </c>
       <c r="R18" s="3" t="n">
@@ -2206,29 +2206,29 @@
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>Signage manufacturer using laser cutting for metal letters, typical buyer of entry-level Chinese fiber lasers.</t>
+          <t>Italian tube laser specialist, could integrate Chinese laser sources for cost-effective tube cutting systems.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Laserage Technology Corporation</t>
+          <t>Signs &amp; Blanks, Inc.</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://www.laserage.com</t>
+          <t>https://www.signsandblanks.com</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>沃基根（Waukegan），伊利诺伊州，美国</t>
+          <t>俄亥俄州托莱多，美国</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2238,27 +2238,27 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>约4000万美元</t>
+          <t>2500万美元</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>提供合同制激光精密加工服务，包括激光切割、焊接、钻孔、刻字，服务医疗器件、电子及航空航天客户。</t>
+          <t>专业生产各类标识标牌、铭牌、控制面板及精密蚀刻零部件，服务于汽车、家电及工业设备行业。</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>高精度纳秒/皮秒激光器（用于微加工）、激光光束传输光学组件、精密运动平台（XY轴）、视觉定位系统。</t>
+          <t>需要采购高精度光纤激光切割机、激光打标机及精密蚀刻设备，用于金属和非金属标牌的高效加工。</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供小批量、多品种快速交付的中国激光器及光学配件供应商，支持定制波长和功率。</t>
+          <t>寻求具备稳定品质、快速交货能力，且能提供定制化激光加工解决方案的中国设备制造商。</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>美国、墨西哥、加拿大、德国、瑞士</t>
+          <t>美国、加拿大、墨西哥、英国</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -2268,22 +2268,22 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Laser Mechanisms、Micron Laser Technology、Laserod</t>
+          <t>Aurora Specialty Products, Inc.、Metalcraft, Inc.、C&amp;H Label</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>美国中西部激光合同加工市场占有率约5%，专注医疗微加工细分领域。</t>
+          <t>北美标识标牌细分市场份额约3%，以汽车OEM铭牌见长。</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2025年新增一台5轴皮秒激光加工中心，用于心脏支架微孔加工，并通过FDA二级医疗器械审核。</t>
+          <t>2025年计划投资100万美元升级激光切割产线，以应对新能源车标识需求增长。</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Job shops &amp; contract manufacturers</t>
+          <t>Signage &amp; metal product companies</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2296,84 +2296,84 @@
           <t>Small (&lt;100)</t>
         </is>
       </c>
-      <c r="R19" s="5" t="n">
-        <v>65</v>
+      <c r="R19" s="3" t="n">
+        <v>70</v>
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>Specialized laser job shop, could add Chinese marking/welding equipment for high-mix low-volume work.</t>
+          <t>Signage manufacturer using laser cutting for metal letters, typical buyer of entry-level Chinese fiber lasers.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Laser Process (UK) Ltd</t>
+          <t>Laserage Technology Corporation</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://www.laserprocess.co.uk</t>
+          <t>https://www.laserage.com</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>伯明翰，英国</t>
+          <t>沃基根（Waukegan），伊利诺伊州，美国</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>约80人</t>
+          <t>120</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>约1500万英镑</t>
+          <t>约4000万美元</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>英国专业激光精密加工服务商，提供激光切割、焊接、打标及微加工服务，服务于航空航天、医疗和电子行业。</t>
+          <t>提供合同制激光精密加工服务，包括激光切割、焊接、钻孔、刻字，服务医疗器件、电子及航空航天客户。</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>采购高精度光纤激光切割头、纳秒/皮秒激光器（用于微加工）、激光焊接视觉定位系统，以及精密运动控制平台。</t>
+          <t>高精度纳秒/皮秒激光器（用于微加工）、激光光束传输光学组件、精密运动平台（XY轴）、视觉定位系统。</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供中小功率（≤500W）高稳定性激光器、具备航空/医疗认证（AS9100/ISO13485）配套经验的中国核心器件供应商。</t>
+          <t>寻找能提供小批量、多品种快速交付的中国激光器及光学配件供应商，支持定制波长和功率。</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>英国、德国、法国、荷兰、瑞士</t>
+          <t>美国、墨西哥、加拿大、德国、瑞士</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>暂无（通过分销商采购激光器）</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Lasertec、TLS Technik、Cutlite Penta</t>
+          <t>Laser Mechanisms、Micron Laser Technology、Laserod</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>英国本地精密激光加工服务市场份额约5%，专注高端利基市场。</t>
+          <t>美国中西部激光合同加工市场占有率约5%，专注医疗微加工细分领域。</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2025年获得英国航天局资助，开发用于卫星部件的高可靠性激光焊接工艺。</t>
+          <t>2025年新增一台5轴皮秒激光加工中心，用于心脏支架微孔加工，并通过FDA二级医疗器械审核。</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
@@ -2396,79 +2396,79 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>UK laser job shop offering cutting/welding, could upgrade with Chinese fiber lasers for cost advantage.</t>
+          <t>Specialized laser job shop, could add Chinese marking/welding equipment for high-mix low-volume work.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Metallurgical Corporation of America (Metco)</t>
+          <t>Laser Process (UK) Ltd</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>https://www.metco.com</t>
+          <t>https://www.laserprocess.co.uk</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>1989</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>休斯顿，美国</t>
+          <t>伯明翰，英国</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>约80人</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>约1.2亿美元</t>
+          <t>约1500万英镑</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>提供金属粉末、热喷涂设备及精密金属零部件加工服务，服务于航空航天、石油天然气及医疗植入物行业。</t>
+          <t>英国专业激光精密加工服务商，提供激光切割、焊接、打标及微加工服务，服务于航空航天、医疗和电子行业。</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>激光熔覆/3D打印用金属粉末（镍基、钴基）、高精度激光焊接设备、真空热处理炉配件。</t>
+          <t>采购高精度光纤激光切割头、纳秒/皮秒激光器（用于微加工）、激光焊接视觉定位系统，以及精密运动控制平台。</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>需要具备粉末冶金或激光增材制造经验的中国供应商，要求提供材料成分检测报告和批量一致性保证。</t>
+          <t>寻找能提供中小功率（≤500W）高稳定性激光器、具备航空/医疗认证（AS9100/ISO13485）配套经验的中国核心器件供应商。</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>美国、加拿大、英国、新加坡、阿联酋</t>
+          <t>英国、德国、法国、荷兰、瑞士</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>暂无（通过分销商采购激光器）</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>欧瑞康美科（Oerlikon Metco）、普莱克斯（Praxair）、Höganäs</t>
+          <t>Lasertec、TLS Technik、Cutlite Penta</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>北美热喷涂粉末市场份额约8%，专注高端定制牌号。</t>
+          <t>英国本地精密激光加工服务市场份额约5%，专注高端利基市场。</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2025年获得美国国防部合同，为海军舰艇提供激光熔覆修复镍基粉末。</t>
+          <t>2025年获得英国航天局资助，开发用于卫星部件的高可靠性激光焊接工艺。</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
@@ -2487,63 +2487,63 @@
         </is>
       </c>
       <c r="R21" s="5" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>US job shop with laser cutting services, likely to consider Chinese machines for cost savings.</t>
+          <t>UK laser job shop offering cutting/welding, could upgrade with Chinese fiber lasers for cost advantage.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Mayer Tool &amp; Manufacturing, Inc.</t>
+          <t>Metallurgical Corporation of America (Metco)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>https://www.mayertool.com</t>
+          <t>https://www.metco.com</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>1965</t>
+          <t>1989</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>伊利诺伊州芝加哥，美国</t>
+          <t>休斯顿，美国</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>350</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>1800万美元</t>
+          <t>约1.2亿美元</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>提供精密金属冲压、CNC加工、工装夹具制造及小批量高精度零部件定制服务，主要服务航空航天和医疗设备客户。</t>
+          <t>提供金属粉末、热喷涂设备及精密金属零部件加工服务，服务于航空航天、石油天然气及医疗植入物行业。</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>需要采购高精度数控磨床、五轴加工中心、激光微加工设备及精密测量仪器，以提升复杂零件加工能力。</t>
+          <t>激光熔覆/3D打印用金属粉末（镍基、钴基）、高精度激光焊接设备、真空热处理炉配件。</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>寻找拥有ISO 13485/AS9100认证，擅长小批量多品种柔性生产，且能配合严格公差要求的中国精密加工设备供应商。</t>
+          <t>需要具备粉末冶金或激光增材制造经验的中国供应商，要求提供材料成分检测报告和批量一致性保证。</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>美国、德国、日本、瑞士</t>
+          <t>美国、加拿大、英国、新加坡、阿联酋</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2553,17 +2553,17 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Proto Labs, Inc.、Xometry, Inc.、Harvey Performance Company</t>
+          <t>欧瑞康美科（Oerlikon Metco）、普莱克斯（Praxair）、Höganäs</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>美国中西部精密加工细分市场占有率约1.2%，聚焦医疗/航空小批量订单。</t>
+          <t>北美热喷涂粉末市场份额约8%，专注高端定制牌号。</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2025年初获得FDA医疗器械合同，计划扩充微加工能力。</t>
+          <t>2025年获得美国国防部合同，为海军舰艇提供激光熔覆修复镍基粉末。</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -2582,188 +2582,188 @@
         </is>
       </c>
       <c r="R22" s="5" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>Small contract manufacturer, could invest in Chinese laser marking for part traceability.</t>
+          <t>US job shop with laser cutting services, likely to consider Chinese machines for cost savings.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Salvagnini Italia S.p.A.</t>
+          <t>Mayer Tool &amp; Manufacturing, Inc.</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>https://www.salvagnini.com</t>
+          <t>https://www.mayertool.com</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>1963</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>维琴察（Vicenza），意大利</t>
+          <t>伊利诺伊州芝加哥，美国</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>1800</t>
+          <t>85</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>约4亿欧元</t>
+          <t>1800万美元</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>柔性钣金加工系统专家，提供P4多边折弯中心、L5光纤激光切割机及S4冲剪复合生产线。</t>
+          <t>提供精密金属冲压、CNC加工、工装夹具制造及小批量高精度零部件定制服务，主要服务航空航天和医疗设备客户。</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>高功率光纤激光器、激光切割光学镜片、液压伺服阀、精密模具钢、自动化料库/机器人集成部件。</t>
+          <t>需要采购高精度数控磨床、五轴加工中心、激光微加工设备及精密测量仪器，以提升复杂零件加工能力。</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>寻找具备大型结构件焊接/加工能力、精通欧洲图纸标准、能配合软件联调（MES接口）的中国供应商。</t>
+          <t>寻找拥有ISO 13485/AS9100认证，擅长小批量多品种柔性生产，且能配合严格公差要求的中国精密加工设备供应商。</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>意大利、德国、美国、墨西哥、波兰</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>萨瓦尼尼（中国）有限公司（上海，设有演示中心和备件库）</t>
+          <t>美国、德国、日本、瑞士</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>通快（TRUMPF）、百超（Bystronic）、天田（AMADA）</t>
+          <t>Proto Labs, Inc.、Xometry, Inc.、Harvey Performance Company</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>全球柔性折弯中心市场占有率约35%，为细分领域绝对龙头。</t>
+          <t>美国中西部精密加工细分市场占有率约1.2%，聚焦医疗/航空小批量订单。</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2025年推出P4Xe混合驱动折弯中心，并宣布在苏州建立亚太首个柔性产线体验中心。</t>
+          <t>2025年初获得FDA医疗器械合同，计划扩充微加工能力。</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Sheet metal fabrication shops</t>
+          <t>Job shops &amp; contract manufacturers</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>Small (&lt;100)</t>
         </is>
       </c>
       <c r="R23" s="5" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>Italian sheet metal machinery maker, may use Chinese lasers in lower-tier product lines.</t>
+          <t>Small contract manufacturer, could invest in Chinese laser marking for part traceability.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TRUMPF Werkzeugmaschinen SE + Co. KG</t>
+          <t>Salvagnini Italia S.p.A.</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>https://www.trumpf.com</t>
+          <t>https://www.salvagnini.com</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>1923</t>
+          <t>1963</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Ditzingen, Germany</t>
+          <t>维琴察（Vicenza），意大利</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>18500</t>
+          <t>1800</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>约54亿欧元</t>
+          <t>约4亿欧元</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>全球领先的激光器、激光加工机床及钣金加工设备制造商，提供从激光器到智能工厂解决方案的全套产品。</t>
+          <t>柔性钣金加工系统专家，提供P4多边折弯中心、L5光纤激光切割机及S4冲剪复合生产线。</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>从中国采购激光器核心光学元件、精密机械零部件、钣金机身铸件及自动化配套部件。</t>
+          <t>高功率光纤激光器、激光切割光学镜片、液压伺服阀、精密模具钢、自动化料库/机器人集成部件。</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>寻找具备精密加工能力、通过ISO 9001认证、能配合欧洲质量标准进行联合研发的中国供应商。</t>
+          <t>寻找具备大型结构件焊接/加工能力、精通欧洲图纸标准、能配合软件联调（MES接口）的中国供应商。</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>德国、中国、美国、日本、韩国</t>
+          <t>意大利、德国、美国、墨西哥、波兰</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>通快（中国）有限公司，位于江苏太仓，设有生产、研发和采购中心</t>
+          <t>萨瓦尼尼（中国）有限公司（上海，设有演示中心和备件库）</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>IPG Photonics, Coherent, Amada</t>
+          <t>通快（TRUMPF）、百超（Bystronic）、天田（AMADA）</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>全球激光加工机床市场占有率约20%，欧洲第一</t>
+          <t>全球柔性折弯中心市场占有率约35%，为细分领域绝对龙头。</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2025年推出新一代TruLaser 5000系列，并宣布扩大太仓工厂产能30%。</t>
+          <t>2025年推出P4Xe混合驱动折弯中心，并宣布在苏州建立亚太首个柔性产线体验中心。</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Industrial equipment distributors</t>
+          <t>Sheet metal fabrication shops</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
@@ -2772,83 +2772,83 @@
         </is>
       </c>
       <c r="R24" s="5" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>German laser giant, unlikely to buy Chinese machines but could distribute or partner for low-end models.</t>
+          <t>Italian sheet metal machinery maker, may use Chinese lasers in lower-tier product lines.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Amada Co., Ltd.</t>
+          <t>TRUMPF Werkzeugmaschinen SE + Co. KG</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>https://www.amada.com</t>
+          <t>https://www.trumpf.com</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>1946</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Isehara, Kanagawa, Japan</t>
+          <t>Ditzingen, Germany</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>11000</t>
+          <t>18500</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>约38亿美元</t>
+          <t>约54亿欧元</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>全球领先的钣金加工设备制造商，产品涵盖激光切割机、数控冲床、折弯机及钣金自动化软件系统。</t>
+          <t>全球领先的激光器、激光加工机床及钣金加工设备制造商，提供从激光器到智能工厂解决方案的全套产品。</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>从中国采购激光切割机用精密导轨、齿轮箱、电气元件、钣金外壳及部分中低功率激光器模块。</t>
+          <t>从中国采购激光器核心光学元件、精密机械零部件、钣金机身铸件及自动化配套部件。</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>寻找具备高精度机加工能力、通过日本品质标准（如JIS）认证、能配合小批量多品种生产模式的中国供应商。</t>
+          <t>寻找具备精密加工能力、通过ISO 9001认证、能配合欧洲质量标准进行联合研发的中国供应商。</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>日本、中国、美国、泰国、德国</t>
+          <t>德国、中国、美国、日本、韩国</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>天田（中国）有限公司，位于上海，设有制造工厂和研发中心（江苏）</t>
+          <t>通快（中国）有限公司，位于江苏太仓，设有生产、研发和采购中心</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>TRUMPF, Bystronic, Mazak</t>
+          <t>IPG Photonics, Coherent, Amada</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>全球钣金加工设备市场占有率约12%，亚洲第一</t>
+          <t>全球激光加工机床市场占有率约20%，欧洲第一</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>2026年发布新一代VISION系列光纤激光切割机，并宣布在中国青岛工厂扩大自动化产线。</t>
+          <t>2025年推出新一代TruLaser 5000系列，并宣布扩大太仓工厂产能30%。</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr">
@@ -2867,111 +2867,206 @@
         </is>
       </c>
       <c r="R25" s="5" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>Japanese laser manufacturer, could source components or entry-level machines from China for emerging markets.</t>
+          <t>German laser giant, unlikely to buy Chinese machines but could distribute or partner for low-end models.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>Amada Co., Ltd.</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amada.com</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>1946</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Isehara, Kanagawa, Japan</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>11000</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>约38亿美元</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>全球领先的钣金加工设备制造商，产品涵盖激光切割机、数控冲床、折弯机及钣金自动化软件系统。</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>从中国采购激光切割机用精密导轨、齿轮箱、电气元件、钣金外壳及部分中低功率激光器模块。</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>寻找具备高精度机加工能力、通过日本品质标准（如JIS）认证、能配合小批量多品种生产模式的中国供应商。</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>日本、中国、美国、泰国、德国</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>天田（中国）有限公司，位于上海，设有制造工厂和研发中心（江苏）</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>TRUMPF, Bystronic, Mazak</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>全球钣金加工设备市场占有率约12%，亚洲第一</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>2026年发布新一代VISION系列光纤激光切割机，并宣布在中国青岛工厂扩大自动化产线。</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Industrial equipment distributors</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>Japanese laser manufacturer, could source components or entry-level machines from China for emerging markets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>Mazak Corporation (Yamazaki Mazak)</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>https://www.mazak.com</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>1919</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Niwa-gun, Aichi Prefecture, Japan</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>约10,500人（全球）</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>约50亿美元（集团）</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>全球领先的数控机床（CNC车床、加工中心、激光加工机）制造商，提供从单机到自动化产线及智能制造解决方案（iSMART Factory）。</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>高功率光纤激光器、激光切割头、精密光学镜片、数控系统配件、钣金结构件、精密铸锻件、伺服电机及驱动部件。</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>具备ISO9001/14001认证，拥有精密加工能力（公差±0.005mm以内），能配合JIT交货，有激光设备配套经验或日系客户合作背景的供应商。</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>日本,美国,中国,德国,印度,巴西,泰国</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="K27" s="4" t="inlineStr">
         <is>
           <t>山崎马扎克（中国）有限公司（上海总部），大连、宁夏小巨人机床（银川）设有生产基地，覆盖全国销售服务网络。</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>DMG MORI, Okuma, Trumpf, Amada, Haas Automation, 大族激光（在激光切割领域）</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>全球数控机床市场份额约5-6%（全球前三），激光加工机领域全球前五。</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
         <is>
           <t>2025年，马扎克发布新一代AI自适应控制激光切割系统（MAZATROL SmoothAi），并宣布扩大中国大连工厂的自动化产线产能，以应对新能源汽车零部件加工需求。</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>设备制造商（OEM）</t>
         </is>
       </c>
-      <c r="P26" s="2" t="inlineStr">
+      <c r="P27" s="2" t="inlineStr">
         <is>
           <t>日本</t>
         </is>
       </c>
-      <c r="Q26" s="2" t="inlineStr">
+      <c r="Q27" s="2" t="inlineStr">
         <is>
           <t>大型（年营收&gt;10亿美元）</t>
         </is>
       </c>
-      <c r="R26" s="6" t="n">
+      <c r="R27" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S26" s="2" t="inlineStr">
+      <c r="S27" s="2" t="inlineStr">
         <is>
           <t>中国在光纤激光器、光学元件及精密钣金领域具备成本与供应链优势，马扎克在华工厂有本地化采购需求。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S26"/>
+  <autoFilter ref="A1:S27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>